<commit_message>
docs de planejamento da sprint 13
</commit_message>
<xml_diff>
--- a/docs/sprints/sprint-12/Tarefas_Sprint_12_OSG_para_importacao.xlsx
+++ b/docs/sprints/sprint-12/Tarefas_Sprint_12_OSG_para_importacao.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas Sprint 12" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legenda" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,8 +30,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -40,6 +44,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00125837"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8CBAD"/>
       </patternFill>
     </fill>
   </fills>
@@ -55,7 +74,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -66,6 +85,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -499,32 +540,32 @@
       </c>
     </row>
     <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>12_Sprint_planejamento tributário e contratos agrários</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>12_Sprint_planejamento tributário e contratos agrários</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>PT-01</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Planejamento Tributário: importar o WP e gerar a apresentação</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Mapear abas, linhas e colunas do WP</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Eduardo</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>## O que / por que
 Definir o contrato da primeira versão do WP de Planejamento Tributário. O mapeamento será a fonte única para a importação e para os slides, evitando regras espalhadas pelo código.
@@ -538,52 +579,52 @@
 Cada campo dos slides possui origem, tipo, unidade, regra de validação e formatação definidos, e o contrato pode ser consumido por PT-02 sem nova leitura exploratória do arquivo.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="G2" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>24/08/2026</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>P4 - Sucessão</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>P4.02 Planejamento Tributário ITCMD</t>
         </is>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>12_Sprint_planejamento tributário e contratos agrários</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>12_Sprint_planejamento tributário e contratos agrários</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>PT-02</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Planejamento Tributário: importar o WP e gerar a apresentação</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Importar, validar e persistir o WP</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Eduardo</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>## O que / por que
 Permitir que o Fiscal carregue o WP fixo, valide os resultados calculados e crie uma revisão rastreável ligada ao cliente, à OS e ao arquivo original.
@@ -597,20 +638,20 @@
 Um WP válido gera snapshot igual ao golden-master e ligado a arquivo, checksum e versão do contrato; arquivo incompatível não cria revisão; reimportação preserva a anterior; auditoria, RLS, testes, typecheck, lint e build passam.</t>
         </is>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="G3" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>27/08/2026</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>P4 - Sucessão</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>P4.02 Planejamento Tributário ITCMD</t>
         </is>
@@ -735,32 +776,32 @@
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>12_Sprint_planejamento tributário e contratos agrários</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>12_Sprint_planejamento tributário e contratos agrários</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>SUC-02</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Sucessão: calculadora e apresentação de ITCMD</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>Gerar a apresentação de ITCMD</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Alexandre</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>## O que / por que
 Gerar a apresentação de ITCMD a partir de uma revisão homologada da calculadora, sem repetir o cálculo dentro do gerador.
@@ -774,52 +815,52 @@
 O PPTX abre sem reparos, segue o padrão visual e apresenta participantes e valores iguais à revisão selecionada, com origem e versão registradas.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="G6" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>03/09/2026</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>P4 - Sucessão</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J6" s="6" t="inlineStr">
         <is>
           <t>P4.02 Planejamento Tributário ITCMD</t>
         </is>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>12_Sprint_planejamento tributário e contratos agrários</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>12_Sprint_planejamento tributário e contratos agrários</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>AGR-01</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Contratos rurais de parceria e composse</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Implementar o cadastro de exploração rural</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Alexandre</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>## O que / por que
 Transformar o mockup em cadastro persistido de parceria e composse, reutilizando as fontes cadastrais existentes.
@@ -833,52 +874,52 @@
 Parceria e composse com múltiplas partes, imóveis e origens sobrevivem a reload; percentuais inválidos não persistem; CUD é auditado; RLS bloqueia outro cluster e os consumidores existentes continuam funcionando.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="G7" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>26/08/2026</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>P3 - Instrumentos Agrários</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>P3.03 Contrato de Parceria Rural</t>
         </is>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>12_Sprint_planejamento tributário e contratos agrários</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>12_Sprint_planejamento tributário e contratos agrários</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>AGR-02</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Contratos rurais de parceria e composse</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Gerar o contrato de parceria rural</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Alexandre</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>## O que / por que
 Gerar e versionar o contrato de parceria rural pelo motor documental usando uma exploração cadastrada.
@@ -892,52 +933,52 @@
 O modelo seleciona a parceria correta; partes, imóveis, áreas e percentuais vêm das fontes certas; prévia e DOCX batem com o modelo; versão antiga permanece imutável e a seed não duplica dados.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="G8" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>31/08/2026</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>P3 - Instrumentos Agrários</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J8" s="4" t="inlineStr">
         <is>
           <t>P3.03 Contrato de Parceria Rural</t>
         </is>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>12_Sprint_planejamento tributário e contratos agrários</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>12_Sprint_planejamento tributário e contratos agrários</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>AGR-03</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Contratos rurais de parceria e composse</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Gerar o contrato de composse rural</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>Alexandre</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>## O que / por que
 Gerar e versionar o contrato de composse rural com compossuidores, frações, imóveis, origens e regras próprias.
@@ -951,20 +992,20 @@
 Somente composses válidas são elegíveis; frações fecham 100%; imóveis e origens são renderizados corretamente; prévia e DOCX batem com o modelo; versões antigas e regressões permanecem estáveis.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="G9" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>04/09/2026</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>P3 - Instrumentos Agrários</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J9" s="4" t="inlineStr">
         <is>
           <t>P3.03 Contrato de Parceria Rural</t>
         </is>
@@ -1030,32 +1071,32 @@
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>12_Sprint_planejamento tributário e contratos agrários</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>12_Sprint_planejamento tributário e contratos agrários</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>GES-03</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Notificações e feed dos projetos da OSG</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Registrar eventos OSG no sino e nos feeds</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>Eduardo</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>## O que / por que
 Adicionar sino interno e evento na thread de cada projeto da OS aos três eventos OSG existentes, preservando e-mail e WhatsApp.
@@ -1069,52 +1110,52 @@
 Cada ocorrência gera exatamente uma entrada em todos os projetos da OS e no máximo um sino por participante; retries não duplicam; lote continua agregado e e-mail/WhatsApp não sofrem regressão.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="n">
+      <c r="G11" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>01/09/2026</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>P6 - Gestão de Projeto OSG</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J11" s="4" t="inlineStr">
         <is>
           <t>P6 - Gestão de Projeto OSG</t>
         </is>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>12_Sprint_planejamento tributário e contratos agrários</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>12_Sprint_planejamento tributário e contratos agrários</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>SUC-01A</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Sucessão: calculadora de ITCMD</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Homologar o modelo de cálculo de ITCMD/MT</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>Alexandre</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>## O que / por que
 Transformar o WP de ITCMD/MT em uma especificação determinística e homologada antes de construir o motor.
@@ -1128,52 +1169,52 @@
 Toda saída possui origem e fórmula rastreáveis, divergências estão decididas, entradas e parâmetros estão classificados e os casos de referência foram aprovados.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="n">
+      <c r="G12" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>24/08/2026</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>P4 - Sucessão</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J12" s="4" t="inlineStr">
         <is>
           <t>P4.02 Planejamento Tributário ITCMD</t>
         </is>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>12_Sprint_planejamento tributário e contratos agrários</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>12_Sprint_planejamento tributário e contratos agrários</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>SUC-01B</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Sucessão: calculadora de ITCMD</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Implementar o domínio e o motor da simulação</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Alexandre</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>## O que / por que
 Implementar o domínio versionado e o motor puro da simulação de ITCMD/MT sem depender do Excel em tempo de execução.
@@ -1187,52 +1228,52 @@
 O motor reproduz os casos homologados com o arredondamento definido, recusa estados inválidos e mantém rastreabilidade e reprodução de cada revisão.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="n">
+      <c r="G13" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>27/08/2026</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>P4 - Sucessão</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J13" s="4" t="inlineStr">
         <is>
           <t>P4.02 Planejamento Tributário ITCMD</t>
         </is>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>12_Sprint_planejamento tributário e contratos agrários</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>12_Sprint_planejamento tributário e contratos agrários</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>SUC-01C</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Sucessão: calculadora de ITCMD</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Entregar a experiência da calculadora</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>Alexandre</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>## O que / por que
 Entregar a interface para montar, comparar, revisar e aprovar simulações de ITCMD usando o motor homologado.
@@ -1246,52 +1287,52 @@
 Um caso homologado é montado e aprovado sem planilha; inconsistências impedem aprovação; a revisão aprovada fica disponível para SUC-02, AC-02 e SUC-03.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="n">
+      <c r="G14" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>31/08/2026</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>P4 - Sucessão</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr">
         <is>
           <t>P4.02 Planejamento Tributário ITCMD</t>
         </is>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>12_Sprint_planejamento tributário e contratos agrários</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>12_Sprint_planejamento tributário e contratos agrários</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>SUC-03A</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>Sucessão: testamento</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>Homologar o caminho e o modelo de testamento</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>Alexandre</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t>## O que / por que
 Definir a modalidade testamentária inicial e quando ela é usada como caminho alternativo à doação em vida.
@@ -1305,52 +1346,52 @@
 Cada variável e condição possui origem definida, a hipótese de uso está clara e existe documento de referência homologado para a implementação.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="n">
+      <c r="G15" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H15" s="8" t="inlineStr">
         <is>
           <t>01/09/2026</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="I15" s="8" t="inlineStr">
         <is>
           <t>P4 - Sucessão</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="J15" s="8" t="inlineStr">
         <is>
           <t>P4.02 Planejamento Tributário ITCMD</t>
         </is>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>12_Sprint_planejamento tributário e contratos agrários</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>12_Sprint_planejamento tributário e contratos agrários</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>SUC-03B</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>Sucessão: testamento</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>Gerar o testamento pelo motor documental</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>Alexandre</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>## O que / por que
 Gerar e versionar o testamento homologado a partir da revisão sucessória escolhida e dos complementos jurídicos.
@@ -1364,52 +1405,52 @@
 O caso golden-master gera documento completo sem ajuste manual, com pessoas, bens, percentuais e disposições iguais à revisão selecionada e histórico preservado.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="n">
+      <c r="G16" s="8" t="n">
         <v>24</v>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H16" s="8" t="inlineStr">
         <is>
           <t>04/09/2026</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="I16" s="8" t="inlineStr">
         <is>
           <t>P4 - Sucessão</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J16" s="8" t="inlineStr">
         <is>
           <t>P4.02 Planejamento Tributário ITCMD</t>
         </is>
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>12_Sprint_planejamento tributário e contratos agrários</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>12_Sprint_planejamento tributário e contratos agrários</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>GES-01A</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Alertas gerenciais automáticos</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Alertar tarefas atrasadas e próximas do prazo</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>Eduardo</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F17" s="5" t="inlineStr">
         <is>
           <t>## O que / por que
 Alertar no sino sobre tarefas abertas próximas do prazo ou atrasadas, sem duplicar o aviso 9 da Sprint 11.
@@ -1423,52 +1464,52 @@
 Cada tarefa gera no máximo um aviso por marco; tarefa resolvida deixa de aparecer; mudança de prazo não mantém alerta falso e o link abre a tarefa correta.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="n">
+      <c r="G17" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>25/08/2026</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>P6 - Gestão de Projeto OSG</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="J17" s="4" t="inlineStr">
         <is>
           <t>P6 - Gestão de Projeto OSG</t>
         </is>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>12_Sprint_planejamento tributário e contratos agrários</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>12_Sprint_planejamento tributário e contratos agrários</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>GES-01B</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>Alertas gerenciais automáticos</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>Alertar inatividade de projetos e tarefas</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>Eduardo</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="F18" s="7" t="inlineStr">
         <is>
           <t>## O que / por que
 Detectar projeto ou tarefa aberta sem movimentação relevante e criar uma ocorrência acionável no sino do gestor.
@@ -1482,52 +1523,52 @@
 A data de última movimentação é explicável; concluídos, cancelados e pausados não alertam; a ocorrência não repete sem mudança e pode nascer novamente após atividade válida.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="n">
+      <c r="G18" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H18" s="6" t="inlineStr">
         <is>
           <t>27/08/2026</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="I18" s="6" t="inlineStr">
         <is>
           <t>P6 - Gestão de Projeto OSG</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="J18" s="6" t="inlineStr">
         <is>
           <t>P6 - Gestão de Projeto OSG</t>
         </is>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>12_Sprint_planejamento tributário e contratos agrários</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>12_Sprint_planejamento tributário e contratos agrários</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>GES-02</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>Alertas gerenciais automáticos</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>Enviar resumo semanal aos gestores</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>Alexandre</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="F19" s="7" t="inlineStr">
         <is>
           <t>## O que / por que
 Enviar um único resumo semanal em e-mail HTML para cada gestor com as pendências do seu escopo.
@@ -1541,52 +1582,52 @@
 Cada gestor recebe no máximo um e-mail por período, com itens e contagens conferidos, links úteis e falhas reprocessáveis sem duplicação.</t>
         </is>
       </c>
-      <c r="G19" s="2" t="n">
+      <c r="G19" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="I19" s="6" t="inlineStr">
         <is>
           <t>P6 - Gestão de Projeto OSG</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="J19" s="6" t="inlineStr">
         <is>
           <t>P6 - Gestão de Projeto OSG</t>
         </is>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>12_Sprint_planejamento tributário e contratos agrários</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>12_Sprint_planejamento tributário e contratos agrários</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>GES-04</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Comunicação automática com clientes</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>Cobrar solicitações sem resposta</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>Alexandre</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>## O que / por que
 Cobrar automaticamente por e-mail e, quando disponível, WhatsApp, as pendências de uma solicitação sem resposta.
@@ -1600,20 +1641,20 @@
 Há no máximo uma comunicação consolidada por marco, destinatário e canal; atividade aprovada interrompe ou recalcula a régua; concorrência e retry não duplicam e o histórico identifica cada envio.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="n">
+      <c r="G20" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>03/09/2026</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="I20" s="4" t="inlineStr">
         <is>
           <t>P6 - Gestão de Projeto OSG</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="J20" s="4" t="inlineStr">
         <is>
           <t>P6 - Gestão de Projeto OSG</t>
         </is>
@@ -1738,32 +1779,32 @@
       </c>
     </row>
     <row r="23" ht="28" customHeight="1">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>12_Sprint_planejamento tributário e contratos agrários</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>12_Sprint_planejamento tributário e contratos agrários</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>AC-01A</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Alterações contratuais por mudanças cadastrais</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>Estruturar o fluxo comum de Alteração Contratual</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>Bernardo</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t>## O que / por que
 Criar a estrutura comum de uma revisão de Alteração Contratual ligada ao instrumento anterior, sem tentar detectar qualquer mudança cadastral automaticamente.
@@ -1777,20 +1818,20 @@
 Uma revisão identifica instrumento, estado-base, mudanças e estado proposto; o estado-base é imutável e o contrato suporta adicionar eventos sem redesenhar a linhagem.</t>
         </is>
       </c>
-      <c r="G23" s="2" t="n">
+      <c r="G23" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="H23" s="4" t="inlineStr">
         <is>
           <t>24/08/2026</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr">
+      <c r="I23" s="4" t="inlineStr">
         <is>
           <t>P2 - Organização Societária</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="J23" s="4" t="inlineStr">
         <is>
           <t>P2.01 Qualificação dos Sócios (WP Sócios + Capital Social)</t>
         </is>
@@ -1915,32 +1956,32 @@
       </c>
     </row>
     <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>12_Sprint_planejamento tributário e contratos agrários</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>12_Sprint_planejamento tributário e contratos agrários</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>AC-03A</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>Alterações contratuais da Agro</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>Homologar os eventos e casos da AC Agro</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>Bernardo</t>
         </is>
       </c>
-      <c r="F26" s="3" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>## O que / por que
 Separar integralização, concentração de cotas, imóvel adicional e exigência cartorial em eventos juridicamente distintos antes da implementação.
@@ -1954,52 +1995,52 @@
 Cada evento possui estado anterior/posterior, dados e gaps identificados, nome não ambíguo e ao menos um caso pequeno priorizado para implementação.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="n">
+      <c r="G26" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H26" s="4" t="inlineStr">
         <is>
           <t>25/08/2026</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="I26" s="4" t="inlineStr">
         <is>
           <t>P2 - Organização Societária</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="J26" s="4" t="inlineStr">
         <is>
           <t>P2.02 Constituição Societária Agro</t>
         </is>
       </c>
     </row>
     <row r="27" ht="28" customHeight="1">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>12_Sprint_planejamento tributário e contratos agrários</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>12_Sprint_planejamento tributário e contratos agrários</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>AC-03B</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>Alterações contratuais da Agro</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>Gerar AC de integralização homologada</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>Bernardo</t>
         </is>
       </c>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="F27" s="5" t="inlineStr">
         <is>
           <t>## O que / por que
 Gerar uma Alteração Contratual de integralização para uma forma de aporte e um caso Agro homologados.
@@ -2013,52 +2054,52 @@
 Capital anterior, aumento, capital posterior, quotas e aportes fecham; cada origem é rastreável e resolução, quadro e consolidado usam os mesmos valores.</t>
         </is>
       </c>
-      <c r="G27" s="2" t="n">
+      <c r="G27" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="H27" s="4" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="I27" s="4" t="inlineStr">
         <is>
           <t>P2 - Organização Societária</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
+      <c r="J27" s="4" t="inlineStr">
         <is>
           <t>P2.02 Constituição Societária Agro</t>
         </is>
       </c>
     </row>
     <row r="28" ht="28" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>12_Sprint_planejamento tributário e contratos agrários</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>12_Sprint_planejamento tributário e contratos agrários</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>AC-03C</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>Alterações contratuais da Agro</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>Gerar AC de concentração de cotas</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t>Bernardo</t>
         </is>
       </c>
-      <c r="F28" s="3" t="inlineStr">
+      <c r="F28" s="5" t="inlineStr">
         <is>
           <t>## O que / por que
 Gerar Alteração Contratual para uma forma homologada de concentração de cotas.
@@ -2072,52 +2113,52 @@
 A soma de quotas é preservada, origem e participantes são rastreáveis, cláusulas condicionais estão corretas e o caso real sai sem edição manual.</t>
         </is>
       </c>
-      <c r="G28" s="2" t="n">
+      <c r="G28" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="H28" s="4" t="inlineStr">
         <is>
           <t>31/08/2026</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
+      <c r="I28" s="4" t="inlineStr">
         <is>
           <t>P2 - Organização Societária</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="J28" s="4" t="inlineStr">
         <is>
           <t>P2.02 Constituição Societária Agro</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>12_Sprint_planejamento tributário e contratos agrários</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>12_Sprint_planejamento tributário e contratos agrários</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>AC-03D</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>Alterações contratuais da Agro</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>Tratar exigência cartorial como revisão</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E29" s="4" t="inlineStr">
         <is>
           <t>Bernardo</t>
         </is>
       </c>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="F29" s="5" t="inlineStr">
         <is>
           <t>## O que / por que
 Tratar exigência cartorial como nova revisão ligada ao documento protocolado, sem sobrescrever o instrumento anterior.
@@ -2131,52 +2172,52 @@
 O documento protocolado permanece imutável; a nova versão identifica exigência e mudanças; prazo e estado são rastreáveis e reexigência não apaga o ciclo anterior.</t>
         </is>
       </c>
-      <c r="G29" s="2" t="n">
+      <c r="G29" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="H29" s="4" t="inlineStr">
         <is>
           <t>02/09/2026</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
+      <c r="I29" s="4" t="inlineStr">
         <is>
           <t>P2 - Organização Societária</t>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr">
+      <c r="J29" s="4" t="inlineStr">
         <is>
           <t>P2.02 Constituição Societária Agro</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>12_Sprint_planejamento tributário e contratos agrários</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>12_Sprint_planejamento tributário e contratos agrários</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>SLD-01A</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C30" s="8" t="inlineStr">
         <is>
           <t>Biblioteca de Slides</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D30" s="8" t="inlineStr">
         <is>
           <t>Estruturar a fundação mínima de templates PPTX</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E30" s="8" t="inlineStr">
         <is>
           <t>Bernardo</t>
         </is>
       </c>
-      <c r="F30" s="3" t="inlineStr">
+      <c r="F30" s="9" t="inlineStr">
         <is>
           <t>## O que / por que
 Criar a fundação mínima e versionada de templates PPTX usada por PT-03 e SUC-02, sem construir editor genérico.
@@ -2190,52 +2231,52 @@
 Todo gerador registra template e versão; versões antigas são imutáveis; template incompatível falha antes do download; fixtures passam pela validação e smoke de abertura, sem regras tributárias na biblioteca comum.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="n">
+      <c r="G30" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="H30" s="8" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr">
+      <c r="I30" s="8" t="inlineStr">
         <is>
           <t>P4 - Sucessão</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr">
+      <c r="J30" s="8" t="inlineStr">
         <is>
           <t>P4.02 Planejamento Tributário ITCMD</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>12_Sprint_planejamento tributário e contratos agrários</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>12_Sprint_planejamento tributário e contratos agrários</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>GOV-01</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>Governança: cadastros da Matriz de Alçadas</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr">
         <is>
           <t>Implementar o cadastro de órgãos de governança</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
         <is>
           <t>Eduardo</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="F31" s="5" t="inlineStr">
         <is>
           <t>## O que / por que
 Entregar o formulário que cadastra as instâncias de decisão de cada cliente, gravando no banco. É ele que define as colunas da Matriz e o destinatário de cada competência no contrato social. Hoje não existe nada: nenhuma tabela de governança está no banco, confirmado por verificação ao vivo em 13/08.
@@ -2249,52 +2290,52 @@
 O consultor abre a tela, cadastra os órgãos de um cliente real, salva, edita e exclui, tudo persistido e auditado, e a tela da Matriz consegue montar suas colunas a partir desse cadastro sem lista fixa em código.</t>
         </is>
       </c>
-      <c r="G31" s="3" t="n">
+      <c r="G31" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="H31" s="3" t="inlineStr">
+      <c r="H31" s="5" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="I31" s="3" t="inlineStr">
+      <c r="I31" s="5" t="inlineStr">
         <is>
           <t>P4 - Governança</t>
         </is>
       </c>
-      <c r="J31" s="3" t="inlineStr">
+      <c r="J31" s="5" t="inlineStr">
         <is>
           <t>Matriz de Alçadas</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>12_Sprint_planejamento tributário e contratos agrários</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>12_Sprint_planejamento tributário e contratos agrários</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
         <is>
           <t>GOV-02</t>
         </is>
       </c>
-      <c r="C32" s="3" t="inlineStr">
+      <c r="C32" s="7" t="inlineStr">
         <is>
           <t>Governança: cadastros da Matriz de Alçadas</t>
         </is>
       </c>
-      <c r="D32" s="3" t="inlineStr">
+      <c r="D32" s="7" t="inlineStr">
         <is>
           <t>Implementar o cadastro da Matriz de Alçadas</t>
         </is>
       </c>
-      <c r="E32" s="3" t="inlineStr">
+      <c r="E32" s="7" t="inlineStr">
         <is>
           <t>Eduardo</t>
         </is>
       </c>
-      <c r="F32" s="3" t="inlineStr">
+      <c r="F32" s="7" t="inlineStr">
         <is>
           <t>## O que / por que
 Entregar a tela em que o consultor preenche a Matriz de Alçadas de um cliente e ela fica gravada. É o documento-eixo da governança e a origem das alíneas de competência de cada órgão na alteração contratual reflexa. Hoje a Matriz existe só como planilha solta por cliente.
@@ -2308,52 +2349,52 @@
 O consultor preenche na tela a matriz de um cliente real do começo ao fim, salva e reabre, com assunto, órgão, papel e alçada persistidos e auditados, e a grade reproduz o modelo VF sem nenhum campo sobrando em texto livre.</t>
         </is>
       </c>
-      <c r="G32" s="3" t="n">
+      <c r="G32" s="7" t="n">
         <v>32</v>
       </c>
-      <c r="H32" s="3" t="inlineStr">
+      <c r="H32" s="7" t="inlineStr">
         <is>
           <t>03/09/2026</t>
         </is>
       </c>
-      <c r="I32" s="3" t="inlineStr">
+      <c r="I32" s="7" t="inlineStr">
         <is>
           <t>P4 - Governança</t>
         </is>
       </c>
-      <c r="J32" s="3" t="inlineStr">
+      <c r="J32" s="7" t="inlineStr">
         <is>
           <t>Matriz de Alçadas</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>12_Sprint_planejamento tributário e contratos agrários</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>12_Sprint_planejamento tributário e contratos agrários</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
         <is>
           <t>GOV-03</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>Governança: cadastros da Matriz de Alçadas</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="D33" s="7" t="inlineStr">
         <is>
           <t>Implementar o cadastro do Acordo de Quotistas</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
+      <c r="E33" s="7" t="inlineStr">
         <is>
           <t>Eduardo</t>
         </is>
       </c>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="F33" s="7" t="inlineStr">
         <is>
           <t>## O que / por que
 Entregar o formulário que grava os parâmetros e os institutos que variam de acordo para acordo. O acordo não é só documento próprio: ele fornece variáveis que a alteração contratual de governança usa, como o limite de aval e fiança em percentual do faturamento, e o usufruto sobre a quota, que decide quem vota e sem o qual qualquer quórum do contrato sai errado.
@@ -2367,22 +2408,372 @@
 O consultor cadastra na tela um acordo real por inteiro, salva e reabre com tudo persistido e auditado, e o sistema sabe, para cada quota gravada com usufruto, quem exerce o direito de voto.</t>
         </is>
       </c>
-      <c r="G33" s="3" t="n">
+      <c r="G33" s="7" t="n">
         <v>24</v>
       </c>
-      <c r="H33" s="3" t="inlineStr">
+      <c r="H33" s="7" t="inlineStr">
         <is>
           <t>08/09/2026</t>
         </is>
       </c>
-      <c r="I33" s="3" t="inlineStr">
+      <c r="I33" s="7" t="inlineStr">
         <is>
           <t>P4 - Governança</t>
         </is>
       </c>
-      <c r="J33" s="3" t="inlineStr">
+      <c r="J33" s="7" t="inlineStr">
         <is>
           <t>Acordo de Quotistas</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="90" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Cor</t>
+        </is>
+      </c>
+      <c r="B1" s="10" t="inlineStr">
+        <is>
+          <t>Significado</t>
+        </is>
+      </c>
+      <c r="C1" s="10" t="inlineStr">
+        <is>
+          <t>Tarefas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Verde</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Concluída (status completed na sprint 12 do Lovable, em 07/09/2026)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>AC-01A, AC-03A, AC-03B, AC-03C, AC-03D, AGR-01, AGR-02, AGR-03, GES-01A, GES-03, GES-04, GOV-01, PT-01, PT-02, SUC-01A, SUC-01B, SUC-01C</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Amarelo</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Citada no texto da semana 1/2 e NÃO concluída (pending ou in_progress)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GES-01B, GES-02, GOV-02, GOV-03, SUC-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Laranja</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Não existe na sprint 12 do Lovable (só na planilha)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>SLD-01A, SUC-03A, SUC-03B</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Sem cor</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Não concluída e não citada no texto das semanas 1/2</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>AC-01B, AC-01C, AC-02, GES-05A, GES-05B, PT-03, PT-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Itens do texto sem tarefa correspondente (nem na planilha, nem com código na sprint 12):</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Eduardo, semana 1</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ajustes no motor para apresentar variáveis</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Alexandre, semana 1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>hotfix para área de solicitação de documentos</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Lovable tem sem código: "3 Auxiliar OSG na Solicitação inicial" (concluída 03/09) e "4 Documento com modelo" (pendente)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Alexandre, semana 1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>RLS</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Bernardo, semana 1</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ACs de variáveis avulsas</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Eduardo, semana 2</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Cadastro do protocolo de remuneração</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Bernardo, semana 2</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>AC de governança</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Tarefas na sprint 12 do Lovable que não estão nesta planilha:</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Corrigir ordenamento das tarefas na PSA projects</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>concluída 04/09</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Permitir editar sub-tarefa a partir da tarefa</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>concluída 04/09</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Botão de projeto restrito (Pausada)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>concluída 28/08</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Auxiliar OSG na Solicitação inicial</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>concluída 03/09</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Documento com modelo: exibir e baixar na solicitação inicial e no portal do cliente</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>pendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>BER-5</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Alterações contratuais e atos societários montados pela biblioteca</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>concluída 01/09</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>BER-6</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Rodar os três recortes candidatos de IA e escolher o da versão 1</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>pendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Suporte PSA</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>pendente</t>
         </is>
       </c>
     </row>

</xml_diff>